<commit_message>
what did i even change?
</commit_message>
<xml_diff>
--- a/Pokedex/Book1.xlsx
+++ b/Pokedex/Book1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dalto\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dalto\Desktop\Repos\PokemonStuff\Pokedex\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4F16990-9AF9-401A-92E1-FCCE22D146F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77676F4B-9A44-4DC6-81CE-54D24C13482C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{0912F9DC-7E4A-4AFD-B84F-FCBF1DC29096}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{0912F9DC-7E4A-4AFD-B84F-FCBF1DC29096}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,13 +35,9 @@
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -70,11 +66,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color indexed="8"/>
-      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="5">
@@ -153,13 +144,13 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -508,60 +499,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:41" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="str">
+      <c r="A1" s="4" t="str">
         <f>_xlfn.CONCAT(A2,"-",F6)</f>
         <v>1-30</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="H1" s="3" t="str">
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="H1" s="4" t="str">
         <f>_xlfn.CONCAT(H2,"-",M6)</f>
         <v>31-60</v>
       </c>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="O1" s="3" t="str">
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="O1" s="4" t="str">
         <f>_xlfn.CONCAT(O2,"-",T6)</f>
         <v>61-90</v>
       </c>
-      <c r="P1" s="3"/>
-      <c r="Q1" s="3"/>
-      <c r="R1" s="3"/>
-      <c r="S1" s="3"/>
-      <c r="T1" s="3"/>
-      <c r="V1" s="3" t="str">
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4"/>
+      <c r="R1" s="4"/>
+      <c r="S1" s="4"/>
+      <c r="T1" s="4"/>
+      <c r="V1" s="4" t="str">
         <f>_xlfn.CONCAT(V2,"-",AA6)</f>
         <v>91-120</v>
       </c>
-      <c r="W1" s="3"/>
-      <c r="X1" s="3"/>
-      <c r="Y1" s="3"/>
-      <c r="Z1" s="3"/>
-      <c r="AA1" s="3"/>
-      <c r="AC1" s="3" t="str">
+      <c r="W1" s="4"/>
+      <c r="X1" s="4"/>
+      <c r="Y1" s="4"/>
+      <c r="Z1" s="4"/>
+      <c r="AA1" s="4"/>
+      <c r="AC1" s="4" t="str">
         <f>_xlfn.CONCAT(AC2,"-",AH6)</f>
         <v>121-150</v>
       </c>
-      <c r="AD1" s="3"/>
-      <c r="AE1" s="3"/>
-      <c r="AF1" s="3"/>
-      <c r="AG1" s="3"/>
-      <c r="AH1" s="3"/>
-      <c r="AJ1" s="3" t="str">
+      <c r="AD1" s="4"/>
+      <c r="AE1" s="4"/>
+      <c r="AF1" s="4"/>
+      <c r="AG1" s="4"/>
+      <c r="AH1" s="4"/>
+      <c r="AJ1" s="4" t="str">
         <f>_xlfn.CONCAT(AJ2,"-",AO6)</f>
         <v>151-180</v>
       </c>
-      <c r="AK1" s="3"/>
-      <c r="AL1" s="3"/>
-      <c r="AM1" s="3"/>
-      <c r="AN1" s="3"/>
-      <c r="AO1" s="3"/>
+      <c r="AK1" s="4"/>
+      <c r="AL1" s="4"/>
+      <c r="AM1" s="4"/>
+      <c r="AN1" s="4"/>
+      <c r="AO1" s="4"/>
     </row>
     <row r="2" spans="1:41" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
@@ -737,7 +728,7 @@
         <f>H2+6</f>
         <v>37</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="3">
         <f t="shared" ref="I3:I6" si="7">I2+6</f>
         <v>38</v>
       </c>
@@ -1294,60 +1285,60 @@
     </row>
     <row r="7" spans="1:41" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="1:41" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="str">
+      <c r="A8" s="4" t="str">
         <f>_xlfn.CONCAT(A9,"-",F13)</f>
         <v>181-210</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="H8" s="3" t="str">
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="H8" s="4" t="str">
         <f>_xlfn.CONCAT(H9,"-",M13)</f>
         <v>211-240</v>
       </c>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="O8" s="3" t="str">
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="O8" s="4" t="str">
         <f>_xlfn.CONCAT(O9,"-",T13)</f>
         <v>241-270</v>
       </c>
-      <c r="P8" s="3"/>
-      <c r="Q8" s="3"/>
-      <c r="R8" s="3"/>
-      <c r="S8" s="3"/>
-      <c r="T8" s="3"/>
-      <c r="V8" s="3" t="str">
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
+      <c r="R8" s="4"/>
+      <c r="S8" s="4"/>
+      <c r="T8" s="4"/>
+      <c r="V8" s="4" t="str">
         <f>_xlfn.CONCAT(V9,"-",AA13)</f>
         <v>271-300</v>
       </c>
-      <c r="W8" s="3"/>
-      <c r="X8" s="3"/>
-      <c r="Y8" s="3"/>
-      <c r="Z8" s="3"/>
-      <c r="AA8" s="3"/>
-      <c r="AC8" s="3" t="str">
+      <c r="W8" s="4"/>
+      <c r="X8" s="4"/>
+      <c r="Y8" s="4"/>
+      <c r="Z8" s="4"/>
+      <c r="AA8" s="4"/>
+      <c r="AC8" s="4" t="str">
         <f>_xlfn.CONCAT(AC9,"-",AH13)</f>
         <v>301-330</v>
       </c>
-      <c r="AD8" s="3"/>
-      <c r="AE8" s="3"/>
-      <c r="AF8" s="3"/>
-      <c r="AG8" s="3"/>
-      <c r="AH8" s="3"/>
-      <c r="AJ8" s="3" t="str">
+      <c r="AD8" s="4"/>
+      <c r="AE8" s="4"/>
+      <c r="AF8" s="4"/>
+      <c r="AG8" s="4"/>
+      <c r="AH8" s="4"/>
+      <c r="AJ8" s="4" t="str">
         <f>_xlfn.CONCAT(AJ9,"-",AO13)</f>
         <v>331-360</v>
       </c>
-      <c r="AK8" s="3"/>
-      <c r="AL8" s="3"/>
-      <c r="AM8" s="3"/>
-      <c r="AN8" s="3"/>
-      <c r="AO8" s="3"/>
+      <c r="AK8" s="4"/>
+      <c r="AL8" s="4"/>
+      <c r="AM8" s="4"/>
+      <c r="AN8" s="4"/>
+      <c r="AO8" s="4"/>
     </row>
     <row r="9" spans="1:41" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -2081,60 +2072,60 @@
     </row>
     <row r="14" spans="1:41" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="15" spans="1:41" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="str">
+      <c r="A15" s="4" t="str">
         <f>_xlfn.CONCAT(A16,"-",F20)</f>
         <v>361-390</v>
       </c>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="H15" s="3" t="str">
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="H15" s="4" t="str">
         <f>_xlfn.CONCAT(H16,"-",M20)</f>
         <v>391-420</v>
       </c>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
-      <c r="O15" s="3" t="str">
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="O15" s="4" t="str">
         <f>_xlfn.CONCAT(O16,"-",T20)</f>
         <v>421-450</v>
       </c>
-      <c r="P15" s="3"/>
-      <c r="Q15" s="3"/>
-      <c r="R15" s="3"/>
-      <c r="S15" s="3"/>
-      <c r="T15" s="3"/>
-      <c r="V15" s="3" t="str">
+      <c r="P15" s="4"/>
+      <c r="Q15" s="4"/>
+      <c r="R15" s="4"/>
+      <c r="S15" s="4"/>
+      <c r="T15" s="4"/>
+      <c r="V15" s="4" t="str">
         <f>_xlfn.CONCAT(V16,"-",AA20)</f>
         <v>451-480</v>
       </c>
-      <c r="W15" s="3"/>
-      <c r="X15" s="3"/>
-      <c r="Y15" s="3"/>
-      <c r="Z15" s="3"/>
-      <c r="AA15" s="3"/>
-      <c r="AC15" s="3" t="str">
+      <c r="W15" s="4"/>
+      <c r="X15" s="4"/>
+      <c r="Y15" s="4"/>
+      <c r="Z15" s="4"/>
+      <c r="AA15" s="4"/>
+      <c r="AC15" s="4" t="str">
         <f>_xlfn.CONCAT(AC16,"-",AH20)</f>
         <v>481-510</v>
       </c>
-      <c r="AD15" s="3"/>
-      <c r="AE15" s="3"/>
-      <c r="AF15" s="3"/>
-      <c r="AG15" s="3"/>
-      <c r="AH15" s="3"/>
-      <c r="AJ15" s="3" t="str">
+      <c r="AD15" s="4"/>
+      <c r="AE15" s="4"/>
+      <c r="AF15" s="4"/>
+      <c r="AG15" s="4"/>
+      <c r="AH15" s="4"/>
+      <c r="AJ15" s="4" t="str">
         <f>_xlfn.CONCAT(AJ16,"-",AO20)</f>
         <v>511-540</v>
       </c>
-      <c r="AK15" s="3"/>
-      <c r="AL15" s="3"/>
-      <c r="AM15" s="3"/>
-      <c r="AN15" s="3"/>
-      <c r="AO15" s="3"/>
+      <c r="AK15" s="4"/>
+      <c r="AL15" s="4"/>
+      <c r="AM15" s="4"/>
+      <c r="AN15" s="4"/>
+      <c r="AO15" s="4"/>
     </row>
     <row r="16" spans="1:41" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
@@ -2868,60 +2859,60 @@
     </row>
     <row r="21" spans="1:41" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="22" spans="1:41" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="3" t="str">
+      <c r="A22" s="4" t="str">
         <f>_xlfn.CONCAT(A23,"-",F27)</f>
         <v>541-570</v>
       </c>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="H22" s="3" t="str">
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="H22" s="4" t="str">
         <f>_xlfn.CONCAT(H23,"-",M27)</f>
         <v>571-600</v>
       </c>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
-      <c r="L22" s="3"/>
-      <c r="M22" s="3"/>
-      <c r="O22" s="3" t="str">
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="4"/>
+      <c r="M22" s="4"/>
+      <c r="O22" s="4" t="str">
         <f>_xlfn.CONCAT(O23,"-",T27)</f>
         <v>601-630</v>
       </c>
-      <c r="P22" s="3"/>
-      <c r="Q22" s="3"/>
-      <c r="R22" s="3"/>
-      <c r="S22" s="3"/>
-      <c r="T22" s="3"/>
-      <c r="V22" s="3" t="str">
+      <c r="P22" s="4"/>
+      <c r="Q22" s="4"/>
+      <c r="R22" s="4"/>
+      <c r="S22" s="4"/>
+      <c r="T22" s="4"/>
+      <c r="V22" s="4" t="str">
         <f>_xlfn.CONCAT(V23,"-",AA27)</f>
         <v>631-660</v>
       </c>
-      <c r="W22" s="3"/>
-      <c r="X22" s="3"/>
-      <c r="Y22" s="3"/>
-      <c r="Z22" s="3"/>
-      <c r="AA22" s="3"/>
-      <c r="AC22" s="3" t="str">
+      <c r="W22" s="4"/>
+      <c r="X22" s="4"/>
+      <c r="Y22" s="4"/>
+      <c r="Z22" s="4"/>
+      <c r="AA22" s="4"/>
+      <c r="AC22" s="4" t="str">
         <f>_xlfn.CONCAT(AC23,"-",AH27)</f>
         <v>661-690</v>
       </c>
-      <c r="AD22" s="3"/>
-      <c r="AE22" s="3"/>
-      <c r="AF22" s="3"/>
-      <c r="AG22" s="3"/>
-      <c r="AH22" s="3"/>
-      <c r="AJ22" s="3" t="str">
+      <c r="AD22" s="4"/>
+      <c r="AE22" s="4"/>
+      <c r="AF22" s="4"/>
+      <c r="AG22" s="4"/>
+      <c r="AH22" s="4"/>
+      <c r="AJ22" s="4" t="str">
         <f>_xlfn.CONCAT(AJ23,"-",AO27)</f>
         <v>691-720</v>
       </c>
-      <c r="AK22" s="3"/>
-      <c r="AL22" s="3"/>
-      <c r="AM22" s="3"/>
-      <c r="AN22" s="3"/>
-      <c r="AO22" s="3"/>
+      <c r="AK22" s="4"/>
+      <c r="AL22" s="4"/>
+      <c r="AM22" s="4"/>
+      <c r="AN22" s="4"/>
+      <c r="AO22" s="4"/>
     </row>
     <row r="23" spans="1:41" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
@@ -3655,60 +3646,60 @@
     </row>
     <row r="28" spans="1:41" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="29" spans="1:41" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="3" t="str">
+      <c r="A29" s="4" t="str">
         <f>_xlfn.CONCAT(A30,"-",F34)</f>
         <v>721-750</v>
       </c>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="3"/>
-      <c r="H29" s="3" t="str">
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="H29" s="4" t="str">
         <f>_xlfn.CONCAT(H30,"-",M34)</f>
         <v>751-780</v>
       </c>
-      <c r="I29" s="3"/>
-      <c r="J29" s="3"/>
-      <c r="K29" s="3"/>
-      <c r="L29" s="3"/>
-      <c r="M29" s="3"/>
-      <c r="O29" s="3" t="str">
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4"/>
+      <c r="L29" s="4"/>
+      <c r="M29" s="4"/>
+      <c r="O29" s="4" t="str">
         <f>_xlfn.CONCAT(O30,"-",T34)</f>
         <v>781-810</v>
       </c>
-      <c r="P29" s="3"/>
-      <c r="Q29" s="3"/>
-      <c r="R29" s="3"/>
-      <c r="S29" s="3"/>
-      <c r="T29" s="3"/>
-      <c r="V29" s="3" t="str">
+      <c r="P29" s="4"/>
+      <c r="Q29" s="4"/>
+      <c r="R29" s="4"/>
+      <c r="S29" s="4"/>
+      <c r="T29" s="4"/>
+      <c r="V29" s="4" t="str">
         <f>_xlfn.CONCAT(V30,"-",AA34)</f>
         <v>811-840</v>
       </c>
-      <c r="W29" s="3"/>
-      <c r="X29" s="3"/>
-      <c r="Y29" s="3"/>
-      <c r="Z29" s="3"/>
-      <c r="AA29" s="3"/>
-      <c r="AC29" s="3" t="str">
+      <c r="W29" s="4"/>
+      <c r="X29" s="4"/>
+      <c r="Y29" s="4"/>
+      <c r="Z29" s="4"/>
+      <c r="AA29" s="4"/>
+      <c r="AC29" s="4" t="str">
         <f>_xlfn.CONCAT(AC30,"-",AH34)</f>
         <v>841-870</v>
       </c>
-      <c r="AD29" s="3"/>
-      <c r="AE29" s="3"/>
-      <c r="AF29" s="3"/>
-      <c r="AG29" s="3"/>
-      <c r="AH29" s="3"/>
-      <c r="AJ29" s="3" t="str">
+      <c r="AD29" s="4"/>
+      <c r="AE29" s="4"/>
+      <c r="AF29" s="4"/>
+      <c r="AG29" s="4"/>
+      <c r="AH29" s="4"/>
+      <c r="AJ29" s="4" t="str">
         <f>_xlfn.CONCAT(AJ30,"-",AO34)</f>
         <v>871-900</v>
       </c>
-      <c r="AK29" s="3"/>
-      <c r="AL29" s="3"/>
-      <c r="AM29" s="3"/>
-      <c r="AN29" s="3"/>
-      <c r="AO29" s="3"/>
+      <c r="AK29" s="4"/>
+      <c r="AL29" s="4"/>
+      <c r="AM29" s="4"/>
+      <c r="AN29" s="4"/>
+      <c r="AO29" s="4"/>
     </row>
     <row r="30" spans="1:41" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
@@ -4442,57 +4433,57 @@
     </row>
     <row r="35" spans="1:41" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="36" spans="1:41" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="3" t="str">
+      <c r="A36" s="4" t="str">
         <f>_xlfn.CONCAT(A37,"-",F41)</f>
         <v>901-930</v>
       </c>
-      <c r="B36" s="3"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="3"/>
-      <c r="E36" s="3"/>
-      <c r="F36" s="3"/>
-      <c r="H36" s="3" t="str">
+      <c r="B36" s="4"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
+      <c r="H36" s="4" t="str">
         <f>_xlfn.CONCAT(H37,"-",M41)</f>
         <v>931-960</v>
       </c>
-      <c r="I36" s="3"/>
-      <c r="J36" s="3"/>
-      <c r="K36" s="3"/>
-      <c r="L36" s="3"/>
-      <c r="M36" s="3"/>
-      <c r="O36" s="3" t="str">
+      <c r="I36" s="4"/>
+      <c r="J36" s="4"/>
+      <c r="K36" s="4"/>
+      <c r="L36" s="4"/>
+      <c r="M36" s="4"/>
+      <c r="O36" s="4" t="str">
         <f>_xlfn.CONCAT(O37,"-",T41)</f>
         <v>961-990</v>
       </c>
-      <c r="P36" s="3"/>
-      <c r="Q36" s="3"/>
-      <c r="R36" s="3"/>
-      <c r="S36" s="3"/>
-      <c r="T36" s="3"/>
-      <c r="V36" s="3" t="str">
+      <c r="P36" s="4"/>
+      <c r="Q36" s="4"/>
+      <c r="R36" s="4"/>
+      <c r="S36" s="4"/>
+      <c r="T36" s="4"/>
+      <c r="V36" s="4" t="str">
         <f>_xlfn.CONCAT(V37,"-",AA41)</f>
         <v>991-1020</v>
       </c>
-      <c r="W36" s="3"/>
-      <c r="X36" s="3"/>
-      <c r="Y36" s="3"/>
-      <c r="Z36" s="3"/>
-      <c r="AA36" s="3"/>
-      <c r="AC36" s="3" t="str">
+      <c r="W36" s="4"/>
+      <c r="X36" s="4"/>
+      <c r="Y36" s="4"/>
+      <c r="Z36" s="4"/>
+      <c r="AA36" s="4"/>
+      <c r="AC36" s="4" t="str">
         <f>_xlfn.CONCAT(AC37,"-",AH41)</f>
         <v>1021-1050</v>
       </c>
-      <c r="AD36" s="3"/>
-      <c r="AE36" s="3"/>
-      <c r="AF36" s="3"/>
-      <c r="AG36" s="3"/>
-      <c r="AH36" s="3"/>
-      <c r="AJ36" s="4"/>
-      <c r="AK36" s="4"/>
-      <c r="AL36" s="4"/>
-      <c r="AM36" s="4"/>
-      <c r="AN36" s="4"/>
-      <c r="AO36" s="4"/>
+      <c r="AD36" s="4"/>
+      <c r="AE36" s="4"/>
+      <c r="AF36" s="4"/>
+      <c r="AG36" s="4"/>
+      <c r="AH36" s="4"/>
+      <c r="AJ36" s="5"/>
+      <c r="AK36" s="5"/>
+      <c r="AL36" s="5"/>
+      <c r="AM36" s="5"/>
+      <c r="AN36" s="5"/>
+      <c r="AO36" s="5"/>
     </row>
     <row r="37" spans="1:41" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
@@ -5106,18 +5097,22 @@
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="AC22:AH22"/>
-    <mergeCell ref="AJ22:AO22"/>
-    <mergeCell ref="AC29:AH29"/>
-    <mergeCell ref="AJ29:AO29"/>
-    <mergeCell ref="AC36:AH36"/>
-    <mergeCell ref="AJ36:AO36"/>
-    <mergeCell ref="AC1:AH1"/>
-    <mergeCell ref="AJ1:AO1"/>
-    <mergeCell ref="AC8:AH8"/>
-    <mergeCell ref="AJ8:AO8"/>
-    <mergeCell ref="AC15:AH15"/>
-    <mergeCell ref="AJ15:AO15"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="H1:M1"/>
+    <mergeCell ref="O1:T1"/>
+    <mergeCell ref="V1:AA1"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="H8:M8"/>
+    <mergeCell ref="O8:T8"/>
+    <mergeCell ref="V8:AA8"/>
+    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="H15:M15"/>
+    <mergeCell ref="O15:T15"/>
+    <mergeCell ref="V15:AA15"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="H22:M22"/>
+    <mergeCell ref="O22:T22"/>
+    <mergeCell ref="V22:AA22"/>
     <mergeCell ref="A29:F29"/>
     <mergeCell ref="H29:M29"/>
     <mergeCell ref="O29:T29"/>
@@ -5126,22 +5121,18 @@
     <mergeCell ref="H36:M36"/>
     <mergeCell ref="O36:T36"/>
     <mergeCell ref="V36:AA36"/>
-    <mergeCell ref="A15:F15"/>
-    <mergeCell ref="H15:M15"/>
-    <mergeCell ref="O15:T15"/>
-    <mergeCell ref="V15:AA15"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="H22:M22"/>
-    <mergeCell ref="O22:T22"/>
-    <mergeCell ref="V22:AA22"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="H1:M1"/>
-    <mergeCell ref="O1:T1"/>
-    <mergeCell ref="V1:AA1"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="H8:M8"/>
-    <mergeCell ref="O8:T8"/>
-    <mergeCell ref="V8:AA8"/>
+    <mergeCell ref="AC1:AH1"/>
+    <mergeCell ref="AJ1:AO1"/>
+    <mergeCell ref="AC8:AH8"/>
+    <mergeCell ref="AJ8:AO8"/>
+    <mergeCell ref="AC15:AH15"/>
+    <mergeCell ref="AJ15:AO15"/>
+    <mergeCell ref="AC22:AH22"/>
+    <mergeCell ref="AJ22:AO22"/>
+    <mergeCell ref="AC29:AH29"/>
+    <mergeCell ref="AJ29:AO29"/>
+    <mergeCell ref="AC36:AH36"/>
+    <mergeCell ref="AJ36:AO36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>